<commit_message>
html and excel report gen
</commit_message>
<xml_diff>
--- a/report.xlsx
+++ b/report.xlsx
@@ -27,11 +27,11 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00008000"/>
+      <color rgb="000000FF"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FF0000"/>
+      <color rgb="00008000"/>
     </font>
     <font>
       <b val="1"/>
@@ -491,81 +491,90 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>test.test_registration</t>
+          <t>test.test_forgot_password</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>test_registration_success</t>
+          <t>test_forgot_password_success</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Verify Register with all valid mandatory fields &amp; unique email.</t>
+          <t>Verify reset password flow for a valid email.</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>SKIPPED</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>21.93053929996677</v>
+        <v>0.0001973002217710018</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-07-23T18:08:03</t>
+          <t>2026-08-13T14:43:57</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Forgot Password API returns 'Account does not exist' for valid accounts in test environment</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>test\test_registration.py</t>
+          <t>test\test_forgot_password.py</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>test/test_registration.py::test_registration_success</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr"/>
+          <t>test/test_forgot_password.py::test_forgot_password_success</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Forgot Password API returns 'Account does not exist' for valid accounts in test environment</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>test.test_registration</t>
+          <t>test.test_forgot_password</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>test_registration_invalid_email[invalidemail]</t>
+          <t>test_forgot_password_invalid_email[unregistered@domain.com]</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Verify email format validation fails with invalid emails.</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
+          <t>Verify forgot password fails with unregistered or invalid email.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>5.544122299877927</v>
+        <v>6.749332600273192</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-07-23T18:08:12</t>
+          <t>2026-08-13T14:44:11</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>test\test_registration.py</t>
+          <t>test\test_forgot_password.py</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>test/test_registration.py::test_registration_invalid_email[invalidemail]</t>
+          <t>test/test_forgot_password.py::test_forgot_password_invalid_email[unregistered@domain.com]</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -573,40 +582,40 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>test.test_registration</t>
+          <t>test.test_forgot_password</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>test_registration_invalid_email[test@.com]</t>
+          <t>test_forgot_password_invalid_email[invalidformat]</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Verify email format validation fails with invalid emails.</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
+          <t>Verify forgot password fails with unregistered or invalid email.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>4.847671400057152</v>
+        <v>6.160873600281775</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-07-23T18:08:20</t>
+          <t>2026-08-13T14:44:17</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>test\test_registration.py</t>
+          <t>test\test_forgot_password.py</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>test/test_registration.py::test_registration_invalid_email[test@.com]</t>
+          <t>test/test_forgot_password.py::test_forgot_password_invalid_email[invalidformat]</t>
         </is>
       </c>
       <c r="J4" t="inlineStr"/>
@@ -614,40 +623,40 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>test.test_registration</t>
+          <t>test.test_forgot_password</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>test_registration_invalid_email[@domain.com]</t>
+          <t>test_forgot_password_blank_email</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Verify email format validation fails with invalid emails.</t>
-        </is>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
+          <t>Verify forgot password handles blank email.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>4.852116399910301</v>
+        <v>6.322298199869692</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-23T18:08:28</t>
+          <t>2026-08-13T14:44:23</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>test\test_registration.py</t>
+          <t>test\test_forgot_password.py</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>test/test_registration.py::test_registration_invalid_email[@domain.com]</t>
+          <t>test/test_forgot_password.py::test_forgot_password_blank_email</t>
         </is>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -655,40 +664,40 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>test.test_registration</t>
+          <t>test.test_login_scenarios</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>test_registration_invalid_email[test@domain]</t>
+          <t>test_login_success</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Verify email format validation fails with invalid emails.</t>
-        </is>
-      </c>
-      <c r="D6" s="1" t="inlineStr">
+          <t>Verify login with valid email and password.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>5.687835100106895</v>
+        <v>25.94482930004597</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-07-23T18:08:37</t>
+          <t>2026-08-13T14:44:49</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>test\test_registration.py</t>
+          <t>test\test_login_scenarios.py</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>test/test_registration.py::test_registration_invalid_email[test@domain]</t>
+          <t>test/test_login_scenarios.py::test_login_success</t>
         </is>
       </c>
       <c r="J6" t="inlineStr"/>
@@ -696,40 +705,40 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>test.test_registration</t>
+          <t>test.test_login_scenarios</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>test_registration_invalid_email[test space@domain.com]</t>
+          <t>test_login_invalid_credentials[nonexistent@domain.com]</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Verify email format validation fails with invalid emails.</t>
-        </is>
-      </c>
-      <c r="D7" s="1" t="inlineStr">
+          <t>Verify login failure with invalid credentials.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>4.892017399892211</v>
+        <v>4.479420700110495</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-07-23T18:08:45</t>
+          <t>2026-08-13T14:44:54</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>test\test_registration.py</t>
+          <t>test\test_login_scenarios.py</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>test/test_registration.py::test_registration_invalid_email[test space@domain.com]</t>
+          <t>test/test_login_scenarios.py::test_login_invalid_credentials[nonexistent@domain.com]</t>
         </is>
       </c>
       <c r="J7" t="inlineStr"/>
@@ -737,40 +746,40 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>test.test_registration</t>
+          <t>test.test_login_scenarios</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>test_registration_blank_mandatory_fields</t>
+          <t>test_login_invalid_credentials[valid@domain.com]</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Register with blank mandatory fields and verify button is disabled or errors show.</t>
-        </is>
-      </c>
-      <c r="D8" s="1" t="inlineStr">
+          <t>Verify login failure with invalid credentials.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>5.621004099957645</v>
+        <v>4.478547600097954</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-07-23T18:08:54</t>
+          <t>2026-08-13T14:44:58</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>test\test_registration.py</t>
+          <t>test\test_login_scenarios.py</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>test/test_registration.py::test_registration_blank_mandatory_fields</t>
+          <t>test/test_login_scenarios.py::test_login_invalid_credentials[valid@domain.com]</t>
         </is>
       </c>
       <c r="J8" t="inlineStr"/>
@@ -778,40 +787,40 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>test.test_registration</t>
+          <t>test.test_login_scenarios</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>test_registration_password_mismatch</t>
+          <t>test_login_security_validation[test@test.com' OR '1'='1]</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Verify password and confirm password match validation.</t>
-        </is>
-      </c>
-      <c r="D9" s="1" t="inlineStr">
+          <t>Verify login handles SQLi and XSS payloads gracefully (Client-side validation).</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.7864744998514652</v>
+        <v>3.711034500040114</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-07-23T18:08:58</t>
+          <t>2026-08-13T14:45:02</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>test\test_registration.py</t>
+          <t>test\test_login_scenarios.py</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>test/test_registration.py::test_registration_password_mismatch</t>
+          <t>test/test_login_scenarios.py::test_login_security_validation[test@test.com' OR '1'='1]</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -819,40 +828,40 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>test.test_registration</t>
+          <t>test.test_login_scenarios</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>test_registration_existing_email</t>
+          <t>test_login_security_validation[&lt;script&gt;alert('xss')&lt;/script&gt;@domain.com]</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Verify existing email address returns appropriate error.</t>
-        </is>
-      </c>
-      <c r="D10" s="1" t="inlineStr">
+          <t>Verify login handles SQLi and XSS payloads gracefully (Client-side validation).</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>8.965031600091606</v>
+        <v>3.331621599849313</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-07-23T18:09:10</t>
+          <t>2026-08-13T14:45:05</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>test\test_registration.py</t>
+          <t>test\test_login_scenarios.py</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>test/test_registration.py::test_registration_existing_email</t>
+          <t>test/test_login_scenarios.py::test_login_security_validation[&lt;script&gt;alert('xss')&lt;/script&gt;@domain.com]</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -860,65 +869,40 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>test.test_forgot_password</t>
+          <t>test.test_login_scenarios</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>test_forgot_password_success</t>
+          <t>test_login_blank_credentials</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Verify reset password flow for a valid email.</t>
+          <t>Verify login with blank email and password.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>FAILED</t>
+          <t>PASSED</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>26.84205099986866</v>
+        <v>4.050427800044417</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-23T18:09:40</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>selenium.common.exceptions.TimeoutException: Message: 
-Stacktrace:
-	chromedriver!GetHandleVerifier [0x7ff6e9c13fa5+14925]
-	chromedriver!GetHandleVerifier [0x7ff6e9c14000+14980]
-	chromedriver!(No symbol) [0x7ff6e975793d]
-	chromedriver!(No symbol) [0x7ff6e97b1aad]
-	chromedriver!(No symbol) [0x7ff6e97b1dac]
-	chromedriver!(No symbol) [0x7ff6e98027d7]
-	chromedriver!(No symbol) [0x7ff6e97ff39b]
-	chromedriver!(No symbol) [0x7ff6e97a401c]
-	chromedriver!(No symbol) [0x7ff6e97a4f43]
-	chromedriver!GetHandleVerifier [0x7ff6ea1f7591+5f7f11]
-	chromedriver!GetHandleVerifier [0x7ff6ea1f1902+5f2282]
-	chromedriver!GetHandleVerifier [0x7ff6ea217115+617a95]
-	chromedriver!GetHandleVerifier [0x7ff6e9c31dce+3274e]
-	chromedriver!GetHandleVerifier [0x7ff6e9c3a82c+3b1ac]
-	chromedriver!GetHandleVerifier [0x7ff6e9c1d744+1e0c4]
-	chromedriver!GetHandleVerifier [0x7ff6e9c1d8d4+1e254]
-	chromedriver!GetHandleVerifier [0x7ff6e9c01447+1dc7]
-	KERNEL32!BaseThreadInitThunk [0x7ffbfff5e957+17]
-	ntdll!RtlUserThreadStart [0x7ffc00bc7c1c+2c]</t>
+          <t>2026-08-13T14:45:09</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>test\test_forgot_password.py</t>
+          <t>test\test_login_scenarios.py</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>test/test_forgot_password.py::test_forgot_password_success</t>
+          <t>test/test_login_scenarios.py::test_login_blank_credentials</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -926,40 +910,40 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>test.test_forgot_password</t>
+          <t>test.test_registration</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>test_forgot_password_invalid_email[unregistered@domain.com]</t>
+          <t>test_registration_success</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Verify forgot password fails with unregistered or invalid email.</t>
-        </is>
-      </c>
-      <c r="D12" s="1" t="inlineStr">
+          <t>Verify Register with all valid mandatory fields &amp; unique email.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>4.356615500058979</v>
+        <v>28.88564449967816</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-07-23T18:09:48</t>
+          <t>2026-08-13T14:45:38</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>test\test_forgot_password.py</t>
+          <t>test\test_registration.py</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>test/test_forgot_password.py::test_forgot_password_invalid_email[unregistered@domain.com]</t>
+          <t>test/test_registration.py::test_registration_success</t>
         </is>
       </c>
       <c r="J12" t="inlineStr"/>
@@ -967,40 +951,40 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>test.test_forgot_password</t>
+          <t>test.test_registration</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>test_forgot_password_invalid_email[invalidformat]</t>
+          <t>test_registration_invalid_email[invalidemail]</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Verify forgot password fails with unregistered or invalid email.</t>
-        </is>
-      </c>
-      <c r="D13" s="1" t="inlineStr">
+          <t>Verify email format validation fails with invalid emails.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>4.451413700124249</v>
+        <v>3.174948699772358</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-07-23T18:09:55</t>
+          <t>2026-08-13T14:45:41</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>test\test_forgot_password.py</t>
+          <t>test\test_registration.py</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>test/test_forgot_password.py::test_forgot_password_invalid_email[invalidformat]</t>
+          <t>test/test_registration.py::test_registration_invalid_email[invalidemail]</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -1008,40 +992,40 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>test.test_forgot_password</t>
+          <t>test.test_registration</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>test_forgot_password_blank_email</t>
+          <t>test_registration_invalid_email[test@.com]</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Verify forgot password handles blank email.</t>
-        </is>
-      </c>
-      <c r="D14" s="1" t="inlineStr">
+          <t>Verify email format validation fails with invalid emails.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>4.535414000041783</v>
+        <v>4.521661499980837</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-07-23T18:10:03</t>
+          <t>2026-08-13T14:45:46</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>test\test_forgot_password.py</t>
+          <t>test\test_registration.py</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>test/test_forgot_password.py::test_forgot_password_blank_email</t>
+          <t>test/test_registration.py::test_registration_invalid_email[test@.com]</t>
         </is>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -1049,40 +1033,40 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>test.test_login_scenarios</t>
+          <t>test.test_registration</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>test_login_success</t>
+          <t>test_registration_invalid_email[@domain.com]</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Verify login with valid email and password.</t>
-        </is>
-      </c>
-      <c r="D15" s="1" t="inlineStr">
+          <t>Verify email format validation fails with invalid emails.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>27.48537169978954</v>
+        <v>3.198782599996775</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-07-23T18:10:34</t>
+          <t>2026-08-13T14:45:50</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>test\test_login_scenarios.py</t>
+          <t>test\test_registration.py</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>test/test_login_scenarios.py::test_login_success</t>
+          <t>test/test_registration.py::test_registration_invalid_email[@domain.com]</t>
         </is>
       </c>
       <c r="J15" t="inlineStr"/>
@@ -1090,40 +1074,40 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>test.test_login_scenarios</t>
+          <t>test.test_registration</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>test_login_invalid_credentials[nonexistent@domain.com]</t>
+          <t>test_registration_invalid_email[test@domain]</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Verify login failure with invalid credentials.</t>
-        </is>
-      </c>
-      <c r="D16" s="1" t="inlineStr">
+          <t>Verify email format validation fails with invalid emails.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>5.983418700052425</v>
+        <v>3.27912380034104</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-07-23T18:10:43</t>
+          <t>2026-08-13T14:45:53</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>test\test_login_scenarios.py</t>
+          <t>test\test_registration.py</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>test/test_login_scenarios.py::test_login_invalid_credentials[nonexistent@domain.com]</t>
+          <t>test/test_registration.py::test_registration_invalid_email[test@domain]</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
@@ -1131,40 +1115,40 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>test.test_login_scenarios</t>
+          <t>test.test_registration</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>test_login_invalid_credentials[valid@domain.com]</t>
+          <t>test_registration_invalid_email[test space@domain.com]</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Verify login failure with invalid credentials.</t>
-        </is>
-      </c>
-      <c r="D17" s="1" t="inlineStr">
+          <t>Verify email format validation fails with invalid emails.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>14.37815660005435</v>
+        <v>4.012023199815303</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-07-23T18:11:00</t>
+          <t>2026-08-13T14:45:57</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>test\test_login_scenarios.py</t>
+          <t>test\test_registration.py</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>test/test_login_scenarios.py::test_login_invalid_credentials[valid@domain.com]</t>
+          <t>test/test_registration.py::test_registration_invalid_email[test space@domain.com]</t>
         </is>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -1172,40 +1156,40 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>test.test_login_scenarios</t>
+          <t>test.test_registration</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>test_login_security_validation[test@test.com' OR '1'='1]</t>
+          <t>test_registration_blank_mandatory_fields</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Verify login handles SQLi and XSS payloads gracefully (Client-side validation).</t>
-        </is>
-      </c>
-      <c r="D18" s="1" t="inlineStr">
+          <t>Register with blank mandatory fields and verify button is disabled or errors show.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>5.847236200002953</v>
+        <v>4.920446600299329</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-07-23T18:11:10</t>
+          <t>2026-08-13T14:46:03</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>test\test_login_scenarios.py</t>
+          <t>test\test_registration.py</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>test/test_login_scenarios.py::test_login_security_validation[test@test.com' OR '1'='1]</t>
+          <t>test/test_registration.py::test_registration_blank_mandatory_fields</t>
         </is>
       </c>
       <c r="J18" t="inlineStr"/>
@@ -1213,40 +1197,40 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>test.test_login_scenarios</t>
+          <t>test.test_registration</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>test_login_security_validation[&lt;script&gt;alert('xss')&lt;/script&gt;@domain.com]</t>
+          <t>test_registration_password_mismatch</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Verify login handles SQLi and XSS payloads gracefully (Client-side validation).</t>
-        </is>
-      </c>
-      <c r="D19" s="1" t="inlineStr">
+          <t>Verify password and confirm password match validation.</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>5.906042900169268</v>
+        <v>2.426638199947774</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-07-23T18:11:19</t>
+          <t>2026-08-13T14:46:05</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>test\test_login_scenarios.py</t>
+          <t>test\test_registration.py</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>test/test_login_scenarios.py::test_login_security_validation[&lt;script&gt;alert('xss')&lt;/script&gt;@domain.com]</t>
+          <t>test/test_registration.py::test_registration_password_mismatch</t>
         </is>
       </c>
       <c r="J19" t="inlineStr"/>
@@ -1254,40 +1238,40 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>test.test_login_scenarios</t>
+          <t>test.test_registration</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>test_login_blank_credentials</t>
+          <t>test_registration_existing_email</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Verify login with blank email and password.</t>
-        </is>
-      </c>
-      <c r="D20" s="1" t="inlineStr">
+          <t>Verify existing email address returns appropriate error.</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>PASSED</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>4.267036900157109</v>
+        <v>8.327043899800628</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-07-23T18:11:26</t>
+          <t>2026-08-13T14:46:14</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>test\test_login_scenarios.py</t>
+          <t>test\test_registration.py</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>test/test_login_scenarios.py::test_login_blank_credentials</t>
+          <t>test/test_registration.py::test_registration_existing_email</t>
         </is>
       </c>
       <c r="J20" t="inlineStr"/>

</xml_diff>